<commit_message>
feat: handlers y rutas de facturación confirmados por el equipo
config-approvers, approval-tray y approvals con sus handlers reales. La ruta
de config-approvers es /api/v1/approvers: tres recursos anidados en el gateway.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lambdas.xlsx
+++ b/lambdas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.fernandez\MEFS-DELOSI\repo_gitlab\ventasCorp-infrastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B538ED25-F27E-4CE2-9CC0-FB37F4CB2A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9502E9C9-63A4-4E3C-8885-71DD9252F0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3976C1CF-DEC9-4EF3-94A9-D9453447DCA5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9F51B622-A81D-425E-8242-25EF68E6B905}"/>
   </bookViews>
   <sheets>
     <sheet name="Lambdas de API" sheetId="1" r:id="rId1"/>
@@ -96,10 +96,10 @@
     <t>Delosi-VentasCorp-Invoicing-Config-Approvers-Lambda-{Env}</t>
   </si>
   <si>
-    <t>/config-approvers</t>
-  </si>
-  <si>
-    <t>Delosi.InvoicingConfigApprovers.Api</t>
+    <t>/api/v1/approvers</t>
+  </si>
+  <si>
+    <t>Delosi.Alfie.Invoicing.ConfigApprover.Api</t>
   </si>
   <si>
     <t>delosi-ventascorp-{env}/invoicing-config-approvers-db
@@ -118,7 +118,7 @@
     <t>/approval-tray</t>
   </si>
   <si>
-    <t>Delosi.InvoicingApprovalTray.Api</t>
+    <t>Delosi.Alfie.Invoicing.ApprovalTray.Api</t>
   </si>
   <si>
     <t>delosi-ventascorp-{env}/invoicing-approval-tray-db
@@ -137,7 +137,7 @@
     <t>/approvals</t>
   </si>
   <si>
-    <t>Delosi.InvoicingApprovals.Api</t>
+    <t>Delosi.Alfie.Invoicing.Approvals.Api</t>
   </si>
   <si>
     <t>delosi-ventascorp-{env}/invoicing-approvals-db
@@ -737,14 +737,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6EA43BA-A7DF-4A81-8A38-C67E778031EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA57D713-19F5-49CE-82A8-FC45CAC5FC18}">
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -1001,7 +1001,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CB9E422-1B9C-4F26-9BFE-AC8A5D361529}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F9F40AD-5D89-4A1A-A5AD-0B44C4C0F5C8}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1144,7 +1144,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C48333A4-5565-4E55-9224-675232AB67ED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E13990E-445B-4F6C-A62C-AAF8B7170A61}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
feat: handlers de sap-sync y notifications confirmados por el equipo
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lambdas.xlsx
+++ b/lambdas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\miguel.fernandez\MEFS-DELOSI\repo_gitlab\ventasCorp-infrastructure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9502E9C9-63A4-4E3C-8885-71DD9252F0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{916295B5-5C87-4739-8117-EC42F1494EC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9F51B622-A81D-425E-8242-25EF68E6B905}"/>
+    <workbookView xWindow="4116" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{303ECDA8-C9E3-4C66-BA06-665FDF160E55}"/>
   </bookViews>
   <sheets>
     <sheet name="Lambdas de API" sheetId="1" r:id="rId1"/>
@@ -269,10 +269,10 @@
     <t>notifications</t>
   </si>
   <si>
-    <t>Delosi.InvoicingNotifications</t>
-  </si>
-  <si>
-    <t>Delosi.InvoicingNotifications.Functions.NotificationFunction</t>
+    <t>Delosi.Alfie.Invoicing.Notifications.Functions</t>
+  </si>
+  <si>
+    <t>Delosi.Alfie.Invoicing.Notifications.Functions.NotificationFunction</t>
   </si>
   <si>
     <t>FunctionHandler</t>
@@ -294,10 +294,10 @@
     <t>sap-sync</t>
   </si>
   <si>
-    <t>Delosi.InvoicingSapSync</t>
-  </si>
-  <si>
-    <t>Delosi.InvoicingSapSync.Functions.SapSyncFunction</t>
+    <t>Delosi.Alfie.Invoicing.SapSync.Functions</t>
+  </si>
+  <si>
+    <t>Delosi.Alfie.Invoicing.SapSync.Functions.SapSyncFunction</t>
   </si>
   <si>
     <t>delosi-ventascorp-{env}/invoicing-sap-sync-db
@@ -737,7 +737,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA57D713-19F5-49CE-82A8-FC45CAC5FC18}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C399819-5FFD-45C2-9138-DFB83782392C}">
   <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1001,14 +1001,14 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F9F40AD-5D89-4A1A-A5AD-0B44C4C0F5C8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{884D2792-4C5C-4280-BF88-2BD45AF1F49F}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -1144,7 +1144,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E13990E-445B-4F6C-A62C-AAF8B7170A61}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811792C7-87F1-4432-9D73-1C554F305C51}">
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>